<commit_message>
Update 3: BIG Update: Added the LaLiga Fantasy page, using the Excel template to import the GW's data, updated tests to test the page.
</commit_message>
<xml_diff>
--- a/collector/templates/laliga-fantasy-oficial.xlsx
+++ b/collector/templates/laliga-fantasy-oficial.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Clubs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Squads'!$A$1:$Q$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Squads'!$A$1:$M$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -502,136 +502,157 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>The official app has no website JSON export. Copy one week at a time from the Android app into this file.</t>
+          <t>The official app starts you with 100M€ and a squad. You buy and sell on the market (or to other managers).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Keep a working copy (for example in Documents). Leave this template in collector/templates/ untouched.</t>
+          <t>There are no captains, vice-captains, or triple captain. The bench is a premium app feature — skip it.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Copy one week at a time from the Android app into this file.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1. Competition — your team name, manager, and season (2026/27).</t>
+          <t>Keep a working copy (for example in Documents). Leave this template in collector/templates/ untouched.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2. Squads — one row per player, every gameweek. Repeat teamPoints / tripleCaptain / transferPenalty on each row of that week.</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>3. Transfers — optional. One row per in/out pair. Skip a week if you made no transfers.</t>
+          <t>1. Competition — your team name, manager, season (2026/27). startingBudget is 100 (not imported).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>4. Clubs — SofaScore club IDs for portraits later. Copy sofaScoreClubId onto Squads/Transfers if you want crests now.</t>
+          <t>2. Squads — every player you own that week. Role starter = Team tab XI. Role squad = Squad tab, not in the XI.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Repeat teamPoints on each row of that week. teamPoints is the app’s week total for the starting XI.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Rules</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>3. Transfers — one row per deal. Bought or Sold, with price and who you traded with (Market or a manager name).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• Do not rename sheets or header cells.</t>
+          <t xml:space="preserve">   Buys and sells are independent. You do not need an in/out pair on the same row.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Delete the yellow EXAMPLE rows before import.</t>
+          <t>4. Clubs — SofaScore club IDs for crests. Copy sofaScoreClubId onto Squads/Transfers if you want crests now.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>• teamPoints is the app’s week total (already includes captain / chips). Do not double it.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>• Captain: TRUE on one starter. Triple captain: TRUE on every row of that week if you played the chip.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Rules</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Positions: GK, DEF, MID, FWD. Roles: starter or bench.</t>
+          <t>• Do not rename sheets or header cells.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• sofaScorePlayerId / sofaScoreClubId are optional. Blank is fine; we can match names later.</t>
+          <t>• Delete the yellow EXAMPLE rows before import.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Positions: GK, DEF, MID, FWD. Roles: starter or squad. No player-count cap — list everyone you own.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Import (from the collector folder, backend running):</t>
+          <t>• Squad-tab players: leave points blank if you cannot see them (premium bench). Price still helps.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python -m collector import-excel templates\laliga-fantasy-oficial.xlsx --dry-run</t>
+          <t>• sofaScorePlayerId / sofaScoreClubId are optional. Blank is fine; we can match names later.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx --gameweek 3</t>
+          <t>Import (from the collector folder, backend running):</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python -m collector import-excel templates\laliga-fantasy-oficial.xlsx --dry-run</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx --gameweek 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>This is a separate competition from SofaScore LaLiga in the dashboard.</t>
         </is>
@@ -649,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -730,6 +751,23 @@
       <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Shown in the dashboard dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>startingBudget</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>App bank at the start of the season, in millions of euros. Not imported.</t>
         </is>
       </c>
     </row>
@@ -745,26 +783,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,130 +824,98 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>tripleCaptain</t>
+          <t>playerName</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>transferPenalty</t>
+          <t>position</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>playerName</t>
+          <t>club</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>role</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>club</t>
+          <t>points</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>rating</t>
         </is>
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>captain</t>
+          <t>price</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
         <is>
-          <t>viceCaptain</t>
+          <t>sofaScorePlayerId</t>
         </is>
       </c>
       <c r="M1" s="4" t="inlineStr">
         <is>
-          <t>points</t>
-        </is>
-      </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="O1" s="4" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="P1" s="4" t="inlineStr">
-        <is>
-          <t>sofaScorePlayerId</t>
-        </is>
-      </c>
-      <c r="Q1" s="4" t="inlineStr">
-        <is>
           <t>sofaScoreClubId</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>GW1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>finished</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="7" t="n">
         <v>64</v>
       </c>
-      <c r="E2" t="b">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>EXAMPLE — delete this row</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>EXAMPLE — starter from Team tab</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>FWD</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Real Madrid</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>starter</t>
         </is>
       </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="I2" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="N2" t="n">
+      <c r="J2" s="7" t="n">
         <v>7.4</v>
       </c>
-      <c r="O2" t="n">
+      <c r="K2" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="L2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -932,69 +934,35 @@
       <c r="D3" s="7" t="n">
         <v>64</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>0</v>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>EXAMPLE — owned, not in XI (Squad tab)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>EXAMPLE — bench placeholder</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>bench</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="N3" s="7" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="O3" s="7" t="n">
+          <t>squad</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="P3" s="7" t="inlineStr"/>
-      <c r="Q3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="n"/>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-    </row>
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4"/>
     <row r="5"/>
     <row r="6"/>
     <row r="7"/>
@@ -1015,26 +983,36 @@
     <row r="22"/>
     <row r="23"/>
     <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
   </sheetData>
-  <autoFilter ref="A1:Q25"/>
-  <dataValidations count="6">
+  <autoFilter ref="A1:M200"/>
+  <dataValidations count="3">
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"finished,live,upcoming"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"GK,DEF,MID,FWD"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
-      <formula1>"starter,bench"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+    <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+      <formula1>"starter,squad"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1048,24 +1026,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1081,67 +1054,42 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>playerIn</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>clubIn</t>
+          <t>playerName</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>positionIn</t>
+          <t>club</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>priceIn</t>
+          <t>position</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>sofaScorePlayerIdIn</t>
+          <t>price</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>sofaScoreClubIdIn</t>
+          <t>counterpart</t>
         </is>
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
-          <t>playerOut</t>
+          <t>sofaScorePlayerId</t>
         </is>
       </c>
       <c r="J1" s="4" t="inlineStr">
         <is>
-          <t>clubOut</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>positionOut</t>
-        </is>
-      </c>
-      <c r="L1" s="4" t="inlineStr">
-        <is>
-          <t>priceOut</t>
-        </is>
-      </c>
-      <c r="M1" s="4" t="inlineStr">
-        <is>
-          <t>sofaScorePlayerIdOut</t>
-        </is>
-      </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>sofaScoreClubIdOut</t>
-        </is>
-      </c>
-      <c r="O1" s="4" t="inlineStr">
-        <is>
-          <t>transferPenalty</t>
+          <t>sofaScoreClubId</t>
         </is>
       </c>
     </row>
@@ -1156,49 +1104,75 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>EXAMPLE — player in</t>
+          <t>Bought</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
+          <t>EXAMPLE — player bought</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
           <t>Real Madrid</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>FWD</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="G2" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr"/>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>EXAMPLE — player out</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>GW2</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Sold</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>EXAMPLE — player sold</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Barcelona</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="L2" s="7" t="n">
+      <c r="G3" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="M2" s="7" t="inlineStr"/>
-      <c r="N2" s="7" t="inlineStr"/>
-      <c r="O2" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3"/>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
+    </row>
     <row r="4"/>
     <row r="5"/>
     <row r="6"/>
@@ -1213,12 +1187,13 @@
     <row r="15"/>
     <row r="16"/>
     <row r="17"/>
+    <row r="18"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
-      <formula1>"GK,DEF,MID,FWD"</formula1>
+    <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+      <formula1>"Bought,Sold"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"GK,DEF,MID,FWD"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update 4: Updated LaLiga Fantasy to include all of the transfers and release clauses and their players that triggered them. Also updated the cmd and all gameweeks for SofaScore Fantasy leagues.
</commit_message>
<xml_diff>
--- a/collector/templates/laliga-fantasy-oficial.xlsx
+++ b/collector/templates/laliga-fantasy-oficial.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -533,7 +533,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>1. Competition — your team name, manager, season (2026/27). startingBudget is 100 (not imported).</t>
+          <t>1. Competition — manager name is enough if the official app has no team name (dashboard will use Locksat).</t>
         </is>
       </c>
     </row>
@@ -568,91 +568,98 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">   channel: Market, or Release clause paid when the other party is a manager (keep counterpart as their name).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>4. Clubs — SofaScore club IDs for crests. Copy sofaScoreClubId onto Squads/Transfers if you want crests now.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>• Do not rename sheets or header cells.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• Delete the yellow EXAMPLE rows before import.</t>
+          <t>• Do not rename sheets or header cells.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• Positions: GK, DEF, MID, FWD. Roles: starter or squad. No player-count cap — list everyone you own.</t>
+          <t>• Delete the yellow EXAMPLE rows before import.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• Squad-tab players: leave points blank if you cannot see them (premium bench). Price still helps.</t>
+          <t>• Positions: GK, DEF, MID, FWD. Roles: starter or squad. No player-count cap — list everyone you own.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>• Squad-tab players: leave points blank if you cannot see them (premium bench). Price still helps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>• sofaScorePlayerId / sofaScoreClubId are optional. Blank is fine; we can match names later.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Import (from the collector folder, backend running):</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python -m collector import-excel templates\laliga-fantasy-oficial.xlsx --dry-run</t>
+          <t>Import (from the collector folder, backend running):</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx</t>
+          <t xml:space="preserve">  python -m collector import-excel templates\laliga-fantasy-oficial.xlsx --dry-run</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  python -m collector import-excel path\to\your-copy.xlsx --gameweek 3</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>This is a separate competition from SofaScore LaLiga in the dashboard.</t>
         </is>
@@ -699,7 +706,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Required. The name shown in the official app.</t>
+          <t>Optional if managerName is set. Official app has no club name; leave blank to use the manager.</t>
         </is>
       </c>
     </row>
@@ -750,7 +757,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Shown in the dashboard dropdown.</t>
+          <t>Shown in the dashboard dropdown. Official private league: El Desafío al Campeón.</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1037,8 +1044,9 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1084,10 +1092,15 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
           <t>sofaScorePlayerId</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>sofaScoreClubId</t>
         </is>
@@ -1130,8 +1143,13 @@
           <t>Market</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr"/>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
       <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -1167,11 +1185,16 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Market</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr"/>
+          <t>Otro Manager FC</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Release clause paid</t>
+        </is>
+      </c>
       <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="inlineStr"/>
     </row>
     <row r="4"/>
     <row r="5"/>
@@ -1189,12 +1212,15 @@
     <row r="17"/>
     <row r="18"/>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Bought,Sold"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"GK,DEF,MID,FWD"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+      <formula1>"Market,Release clause paid"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>